<commit_message>
etapa de produccion / cambio en modal / archivo de carga
</commit_message>
<xml_diff>
--- a/docs/importacion_particulares_2026.xlsx
+++ b/docs/importacion_particulares_2026.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Enrique Arenas\Documents\Control de Entregas - Formatto\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7E87213-E178-4343-B43C-B53E133EE548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98ED2B2B-458F-4BBA-938E-53AAA9B3865B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29610" yWindow="-120" windowWidth="28110" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29610" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carga Mayo" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="138">
   <si>
     <t>Periodo</t>
   </si>
@@ -410,6 +411,30 @@
   </si>
   <si>
     <t>Cubicado | NV: 100091035</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>SODIMAC</t>
+  </si>
+  <si>
+    <t>CONSTRUMART</t>
+  </si>
+  <si>
+    <t>ESTANTE ESCALA</t>
+  </si>
+  <si>
+    <t>REPISA LINEAL 600X300 NEGRO</t>
+  </si>
+  <si>
+    <t>REPISA LINEAL 600X300 BLANCO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VANITORIO REVERSIBLE NOGAL LINCOLN </t>
+  </si>
+  <si>
+    <t>Forecast</t>
   </si>
 </sst>
 </file>
@@ -427,6 +452,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -489,7 +515,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -500,34 +526,16 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF8EC"/>
-          <bgColor rgb="FFFFF8EC"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -976,6 +984,30 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF8EC"/>
+          <bgColor rgb="FFFFF8EC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
@@ -990,7 +1022,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F2B3772-AE31-4B15-905F-8077AFE8F892}" name="Tabla1" displayName="Tabla1" ref="A1:K53" totalsRowShown="0" dataDxfId="0" tableBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F2B3772-AE31-4B15-905F-8077AFE8F892}" name="Tabla1" displayName="Tabla1" ref="A1:K53" totalsRowShown="0" dataDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A1:K53" xr:uid="{2F2B3772-AE31-4B15-905F-8077AFE8F892}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{A65D0286-D9FC-4F7F-93A5-79DE78B9AA2E}" name="Periodo" dataDxfId="11"/>
@@ -1004,6 +1036,26 @@
     <tableColumn id="9" xr3:uid="{C998F1F0-914E-4D9C-8BAC-8629EB0A4C33}" name="Piso" dataDxfId="3"/>
     <tableColumn id="10" xr3:uid="{0A22C010-FFA5-43E7-86AA-977A1AB57420}" name="Deptos/Casas" dataDxfId="2"/>
     <tableColumn id="11" xr3:uid="{B0BA20A0-78C4-4B1A-AC1F-9CA7385262BC}" name="Observacion" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C20AE68E-0472-48ED-AF68-C11E20A804E0}" name="Tabla2" displayName="Tabla2" ref="A1:K19" totalsRowShown="0">
+  <autoFilter ref="A1:K19" xr:uid="{C20AE68E-0472-48ED-AF68-C11E20A804E0}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{85D5102F-6DA2-4AE1-815B-2191FA226D79}" name="Periodo"/>
+    <tableColumn id="2" xr3:uid="{138E1826-A94D-47BD-9BC8-4F482FE6D77F}" name="Linea Negocio"/>
+    <tableColumn id="3" xr3:uid="{ADBCA05E-F73E-4AD0-8C06-3AEA4E15B5C6}" name="Proyecto"/>
+    <tableColumn id="4" xr3:uid="{270AA76F-B400-4285-AD1A-CE9FF47EE1BF}" name="Fecha Despacho"/>
+    <tableColumn id="5" xr3:uid="{E5D53CEF-1D97-4F46-A587-91582E0B31D7}" name="Tipo"/>
+    <tableColumn id="6" xr3:uid="{B40F849C-0071-484D-9507-7BF9FC041E34}" name="Descripcion"/>
+    <tableColumn id="7" xr3:uid="{061C81DD-5AAF-4CD1-AEBE-157C544B929F}" name="Torre"/>
+    <tableColumn id="8" xr3:uid="{0698FAD1-BDFE-4A37-8DA3-82C932A900F8}" name="Nucleo"/>
+    <tableColumn id="9" xr3:uid="{DDC09ACA-55A8-4ADB-80C0-553701524D24}" name="Piso"/>
+    <tableColumn id="10" xr3:uid="{70FEBFFC-2AED-4E9F-BC31-9446F38326E3}" name="Deptos/Casas" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{142BB7CC-DA92-439D-ADFA-8AA3979D8247}" name="Observacion"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2894,4 +2946,528 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D808FECB-B9DB-4B99-8175-BB5A026F5398}">
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.59765625" customWidth="1"/>
+    <col min="3" max="3" width="27.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.296875" customWidth="1"/>
+    <col min="6" max="6" width="12.5" customWidth="1"/>
+    <col min="10" max="10" width="14" style="4" customWidth="1"/>
+    <col min="11" max="11" width="25.09765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>106</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="K3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>109</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="K4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="K5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>111</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>112</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="K8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="K9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>114</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" t="s">
+        <v>118</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="K10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>119</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" t="s">
+        <v>122</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" t="s">
+        <v>124</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K13" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>120</v>
+      </c>
+      <c r="D14" t="s">
+        <v>121</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
+        <v>125</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>126</v>
+      </c>
+      <c r="D15" t="s">
+        <v>127</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>128</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K15" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" t="s">
+        <v>131</v>
+      </c>
+      <c r="D16" t="s">
+        <v>127</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" t="s">
+        <v>133</v>
+      </c>
+      <c r="J16" s="4">
+        <v>200</v>
+      </c>
+      <c r="K16" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" t="s">
+        <v>132</v>
+      </c>
+      <c r="D17" t="s">
+        <v>127</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>134</v>
+      </c>
+      <c r="J17" s="4">
+        <v>100</v>
+      </c>
+      <c r="K17" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" t="s">
+        <v>127</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" t="s">
+        <v>135</v>
+      </c>
+      <c r="J18" s="4">
+        <v>100</v>
+      </c>
+      <c r="K18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" t="s">
+        <v>132</v>
+      </c>
+      <c r="D19" t="s">
+        <v>127</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" t="s">
+        <v>136</v>
+      </c>
+      <c r="J19" s="4">
+        <v>100</v>
+      </c>
+      <c r="K19" t="s">
+        <v>137</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>